<commit_message>
Update construction manual and BOM for battery changes
Updated the ConstructionManual.md and PDF to reflect new LiPo battery specifications and connector type (JST-PH 2.0) effective from January 2026. Added new images for battery and connection instructions, and revised BOM to match updated battery details.
</commit_message>
<xml_diff>
--- a/3D print files/Bill of Material quantum dice.xlsx
+++ b/3D print files/Bill of Material quantum dice.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aernoutvanrossum/Github/Quantum-Dice-by-UTwente/3D print files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5AD8110-FC91-554F-BD39-36809DF21B19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4847193-C6D0-6A41-BF3E-D2E616E83A9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="860" windowWidth="28800" windowHeight="15800" xr2:uid="{281531AD-289F-7444-9810-C417D6306E6A}"/>
   </bookViews>
@@ -2044,6 +2044,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FF458063C0B8354687E7E385217DADDD" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="db0b04aaa15c7297f6f6526469376690">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5f810545-bb7d-498e-98a6-3cc8175571c8" xmlns:ns3="8077f6fe-c9e5-4688-b004-da2992bb8cd8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="66dfeb35f9f6b101ff511922eb62fa51" ns2:_="" ns3:_="">
     <xsd:import namespace="5f810545-bb7d-498e-98a6-3cc8175571c8"/>
@@ -2250,15 +2259,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D196A880-6C6D-4D69-8998-929C3B39CF40}">
   <ds:schemaRefs>
@@ -2277,6 +2277,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CAA44028-4133-420E-8665-60C989F4E89B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BC96DF67-5917-4890-8162-737ED9540272}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2293,12 +2301,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CAA44028-4133-420E-8665-60C989F4E89B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Reorganize 3D print files and update BOM
Clean up and reorganize 3D print assets: moved TPUFrameOnly parts into a new "Version 2" directory (13 files renamed/moved) to consolidate versioned prints, deleted seven obsolete STL files from QuantumDice V2 PrintParts, and updated the Bill of Material spreadsheet (Bill of Material quantum dice.xlsx). This is a repository structure and BOM update to reflect the current Version 2 parts and remove legacy files.
</commit_message>
<xml_diff>
--- a/3D print files/Bill of Material quantum dice.xlsx
+++ b/3D print files/Bill of Material quantum dice.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aernoutvanrossum/Github/Quantum-Dice-by-UTwente/3D print files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E715D3F6-8578-6945-BF91-A5B29485E03A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D4CD169-3843-CD4A-9187-178D13D37E7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11200" yWindow="600" windowWidth="28800" windowHeight="15960" xr2:uid="{281531AD-289F-7444-9810-C417D6306E6A}"/>
+    <workbookView xWindow="11200" yWindow="600" windowWidth="34240" windowHeight="21140" xr2:uid="{281531AD-289F-7444-9810-C417D6306E6A}"/>
   </bookViews>
   <sheets>
-    <sheet name="TPUFrameOnly" sheetId="2" r:id="rId1"/>
+    <sheet name="version2" sheetId="2" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -181,7 +181,7 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Check polarity! If not ok, request swap of polarity through message center
+          <t xml:space="preserve">Check polarity! If not ok, request swap of polarity through message center of Aliexpress
 </t>
         </r>
         <r>
@@ -200,7 +200,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="67">
   <si>
     <t>1.28 inch IPS Color TFT LCD Display Module 1.28" RGB LED Round Touch Screen GC9A01 Drive 4 Wire SPI Interface 240x240 PCB Board</t>
   </si>
@@ -334,9 +334,6 @@
     <t>02A_Yellow_TPU_V*_display_cup_power_USB-C</t>
   </si>
   <si>
-    <t>Frame parts of TPU, with bumper. Cups of PLA</t>
-  </si>
-  <si>
     <t>cable set, containing:</t>
   </si>
   <si>
@@ -398,6 +395,12 @@
   </si>
   <si>
     <t>https://nl.aliexpress.com/item/1005004379893877.html</t>
+  </si>
+  <si>
+    <t>Frame parts of TPU, with bumper. Cups of PLA. Software version &gt; V.2.0.0</t>
+  </si>
+  <si>
+    <t>For version 1.x.x the Blue top cup has an A and B indication</t>
   </si>
 </sst>
 </file>
@@ -903,7 +906,7 @@
         <v>31</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D1" s="5"/>
       <c r="E1" s="2" t="s">
@@ -912,13 +915,18 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C2">
         <v>2</v>
       </c>
       <c r="E2" t="s">
-        <v>44</v>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E3" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -934,7 +942,7 @@
         <v>3</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E9" t="s">
         <v>17</v>
@@ -952,7 +960,7 @@
         <v>1</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
@@ -967,7 +975,7 @@
         <v>1</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
@@ -982,7 +990,7 @@
         <v>2</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
@@ -997,7 +1005,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
@@ -1012,7 +1020,7 @@
         <v>1</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
@@ -1027,12 +1035,12 @@
         <v>2</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B16" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C16">
         <f t="shared" si="0"/>
@@ -1042,7 +1050,7 @@
         <v>2</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.2">
@@ -1057,7 +1065,7 @@
         <v>4</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.2">
@@ -1072,7 +1080,7 @@
         <v>1</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.2">
@@ -1087,7 +1095,7 @@
         <v>1</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.2">
@@ -1154,7 +1162,7 @@
     </row>
     <row r="26" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B26" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C26">
         <f t="shared" si="1"/>
@@ -1164,7 +1172,7 @@
         <v>4</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="28" spans="2:5" x14ac:dyDescent="0.2">
@@ -1219,7 +1227,7 @@
     </row>
     <row r="32" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B32" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C32">
         <f t="shared" si="2"/>
@@ -1234,7 +1242,7 @@
     </row>
     <row r="33" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B33" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C33">
         <f t="shared" si="2"/>
@@ -1244,12 +1252,12 @@
         <v>1</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="34" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B34" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C34">
         <f t="shared" si="2"/>
@@ -1259,15 +1267,15 @@
         <v>1</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="36" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B36" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E36" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="37" spans="2:5" x14ac:dyDescent="0.2">
@@ -1362,12 +1370,12 @@
     </row>
     <row r="43" spans="2:5" x14ac:dyDescent="0.2">
       <c r="E43" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="44" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B44" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C44">
         <v>1</v>
@@ -1388,12 +1396,12 @@
     </row>
     <row r="48" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B48" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="49" spans="2:5" ht="17" x14ac:dyDescent="0.2">
       <c r="B49" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C49">
         <f t="shared" ref="C49:C52" si="4">$C$2*D49</f>
@@ -1407,7 +1415,7 @@
     </row>
     <row r="50" spans="2:5" ht="17" x14ac:dyDescent="0.2">
       <c r="B50" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C50">
         <f t="shared" si="4"/>
@@ -1421,7 +1429,7 @@
     </row>
     <row r="51" spans="2:5" ht="17" x14ac:dyDescent="0.2">
       <c r="B51" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C51">
         <f t="shared" si="4"/>
@@ -1434,7 +1442,7 @@
     </row>
     <row r="52" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B52" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C52">
         <f t="shared" si="4"/>
@@ -1462,14 +1470,35 @@
     <hyperlink ref="E11:E19" r:id="rId13" display="https://github.com/qlab-utwente/Quantum-Dice-by-UTwente/tree/main/3D%20print%20files/quantum%20dice%203D%20print%20parts%20TPUFrameOnly" xr:uid="{F1AB62F5-AC28-0A43-9BB4-0725CAEB4FF4}"/>
     <hyperlink ref="E29" r:id="rId14" xr:uid="{3F271A1C-56E6-A041-9730-1CA5C8FB6613}"/>
     <hyperlink ref="E43" r:id="rId15" xr:uid="{B9C93A19-0F01-0F48-A6FD-83ED74C661E6}"/>
+    <hyperlink ref="E33" r:id="rId16" xr:uid="{E26307DB-87D9-CF49-ACEC-9FF4E814A6D9}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId16"/>
-  <legacyDrawing r:id="rId17"/>
+  <drawing r:id="rId17"/>
+  <legacyDrawing r:id="rId18"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5f810545-bb7d-498e-98a6-3cc8175571c8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="8077f6fe-c9e5-4688-b004-da2992bb8cd8" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FF458063C0B8354687E7E385217DADDD" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="db0b04aaa15c7297f6f6526469376690">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5f810545-bb7d-498e-98a6-3cc8175571c8" xmlns:ns3="8077f6fe-c9e5-4688-b004-da2992bb8cd8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="66dfeb35f9f6b101ff511922eb62fa51" ns2:_="" ns3:_="">
     <xsd:import namespace="5f810545-bb7d-498e-98a6-3cc8175571c8"/>
@@ -1676,41 +1705,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5f810545-bb7d-498e-98a6-3cc8175571c8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="8077f6fe-c9e5-4688-b004-da2992bb8cd8" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BC96DF67-5917-4890-8162-737ED9540272}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CAA44028-4133-420E-8665-60C989F4E89B}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="5f810545-bb7d-498e-98a6-3cc8175571c8"/>
-    <ds:schemaRef ds:uri="8077f6fe-c9e5-4688-b004-da2992bb8cd8"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1733,9 +1731,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CAA44028-4133-420E-8665-60C989F4E89B}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BC96DF67-5917-4890-8162-737ED9540272}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="5f810545-bb7d-498e-98a6-3cc8175571c8"/>
+    <ds:schemaRef ds:uri="8077f6fe-c9e5-4688-b004-da2992bb8cd8"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>